<commit_message>
Rerun eval with 10x size with convergence analysis, starting opt next
</commit_message>
<xml_diff>
--- a/eval/Final_Results.xlsx
+++ b/eval/Final_Results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ian-g8\projects\FinalTop\eval\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ian-g8\projects\FinalTop\eval_10x\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BB0CCA-BAA3-4C07-A389-8D5FB0E30EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B361B9F-E226-47A7-9F08-8A33070D0729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DC97868F-0C32-49C4-BD1D-CDEEAEA189B3}"/>
   </bookViews>
@@ -112,8 +112,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0000"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
@@ -163,15 +162,15 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="15">
     <dxf>
       <font>
         <b val="0"/>
@@ -255,6 +254,18 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <font>
@@ -1079,19 +1090,19 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$B$10:$B$13</c:f>
               <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.8438298034523</c:v>
+                  <c:v>18.421462741213698</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.7286666346497299</c:v>
+                  <c:v>17.266254811593701</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.71755194470252</c:v>
+                  <c:v>17.154739436798899</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.7615745175880899</c:v>
+                  <c:v>17.596416562498199</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1150,19 +1161,19 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$C$10:$C$13</c:f>
               <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.84338246688453</c:v>
+                  <c:v>18.416951952933001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.7287784283543099</c:v>
+                  <c:v>17.267316870122901</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.7178082711451399</c:v>
+                  <c:v>17.157242310400498</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.7614138277217</c:v>
+                  <c:v>17.5947611027206</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1221,19 +1232,19 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$D$10:$D$13</c:f>
               <c:numCache>
-                <c:formatCode>0.0000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1.8487956246572099</c:v>
+                  <c:v>18.475893918431499</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.7359708081387899</c:v>
+                  <c:v>17.345315007912301</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.7251720106530299</c:v>
+                  <c:v>17.237104830960799</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.76809188651991</c:v>
+                  <c:v>17.667195454988001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1453,7 +1464,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.0000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1698,22 +1709,22 @@
             <c:numRef>
               <c:f>Beam_Comparison!$B$3:$B$7</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.132837940797006</c:v>
+                  <c:v>1.3491828990000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.45704881801401098</c:v>
+                  <c:v>4.5914016670000004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.70088400530086803</c:v>
+                  <c:v>7.0140517329999996</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.92486510535883804</c:v>
+                  <c:v>9.2493070320000008</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.43565511996297401</c:v>
+                  <c:v>4.3528580320000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1775,22 +1786,22 @@
             <c:numRef>
               <c:f>Beam_Comparison!$C$3:$C$7</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.71476068422335E-2</c:v>
+                  <c:v>0.47367235699999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.18438431330628</c:v>
+                  <c:v>1.848991979</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.34541796582759698</c:v>
+                  <c:v>3.45726975</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.576477041859215</c:v>
+                  <c:v>5.7607147589999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.43687707375074197</c:v>
+                  <c:v>4.3642715169999997</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1852,22 +1863,22 @@
             <c:numRef>
               <c:f>Beam_Comparison!$D$3:$D$7</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>4.0631446354482598E-2</c:v>
+                  <c:v>0.40781563900000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.159811500172961</c:v>
+                  <c:v>1.6018056789999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.30388583540334402</c:v>
+                  <c:v>3.0412965669999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.52327219067318398</c:v>
+                  <c:v>5.229179222</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.43697983419269099</c:v>
+                  <c:v>4.3652269190000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1929,22 +1940,22 @@
             <c:numRef>
               <c:f>Beam_Comparison!$E$3:$E$7</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>6.7857361094004004E-2</c:v>
+                  <c:v>0.68377695299999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.259349362226998</c:v>
+                  <c:v>2.6036390140000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.46131548553317597</c:v>
+                  <c:v>4.6174345839999997</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.70681956698280002</c:v>
+                  <c:v>7.0634611239999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.43654444642909401</c:v>
+                  <c:v>4.361258791</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2157,7 +2168,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4068,17 +4079,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}" name="Table1" displayName="Table1" ref="A11:D16" totalsRowShown="0" dataDxfId="10" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}" name="Table1" displayName="Table1" ref="A11:D16" totalsRowShown="0" dataDxfId="14" dataCellStyle="Percent">
   <autoFilter ref="A11:D16" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{1C96DD68-5388-41C8-80A4-631AF2530025}" name="Load Case"/>
-    <tableColumn id="2" xr3:uid="{C0C49FD7-8D17-437F-88C8-BB6258B99219}" name="Guth" dataDxfId="9" dataCellStyle="Percent">
+    <tableColumn id="2" xr3:uid="{C0C49FD7-8D17-437F-88C8-BB6258B99219}" name="Guth" dataDxfId="13" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((C3-B3)/B3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{CB5631BD-80FB-4B0B-BC78-3E45F11C5622}" name="Mooney" dataDxfId="8" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{CB5631BD-80FB-4B0B-BC78-3E45F11C5622}" name="Mooney" dataDxfId="12" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((D3-B3)/B3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{64489D84-8154-4AB7-B213-01F3A56C4E26}" name="Kerner" dataDxfId="7" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{64489D84-8154-4AB7-B213-01F3A56C4E26}" name="Kerner" dataDxfId="11" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((E3-B3)/B3)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4091,10 +4102,10 @@
   <autoFilter ref="A2:E7" xr:uid="{1636F957-79EA-4A9C-A088-0551A65C1F5C}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{BBB9A9AD-3816-4FCF-910B-BC91E45978F8}" name="Load Magnitude"/>
-    <tableColumn id="2" xr3:uid="{C2C97874-87BF-4F49-8E77-46CBD4B4BE4A}" name="Default"/>
-    <tableColumn id="3" xr3:uid="{2269703A-CD27-4542-B024-242B1A805057}" name="Guth"/>
-    <tableColumn id="4" xr3:uid="{CF64BBBD-0D58-4197-9737-466E1D604376}" name="Mooney"/>
-    <tableColumn id="5" xr3:uid="{2F62C0DF-5422-48A6-88EC-800D14AC8CAF}" name="Kerner"/>
+    <tableColumn id="2" xr3:uid="{C2C97874-87BF-4F49-8E77-46CBD4B4BE4A}" name="Default" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{2269703A-CD27-4542-B024-242B1A805057}" name="Guth" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{CF64BBBD-0D58-4197-9737-466E1D604376}" name="Mooney" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{2F62C0DF-5422-48A6-88EC-800D14AC8CAF}" name="Kerner" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4427,7 +4438,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -4502,7 +4513,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4524,60 +4535,60 @@
       <c r="A10" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="1">
-        <v>1.8438298034523</v>
-      </c>
-      <c r="C10" s="1">
-        <v>1.84338246688453</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1.8487956246572099</v>
+      <c r="B10">
+        <v>18.421462741213698</v>
+      </c>
+      <c r="C10">
+        <v>18.416951952933001</v>
+      </c>
+      <c r="D10">
+        <v>18.475893918431499</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="1">
-        <v>1.7286666346497299</v>
-      </c>
-      <c r="C11" s="1">
-        <v>1.7287784283543099</v>
-      </c>
-      <c r="D11" s="1">
-        <v>1.7359708081387899</v>
+      <c r="B11">
+        <v>17.266254811593701</v>
+      </c>
+      <c r="C11">
+        <v>17.267316870122901</v>
+      </c>
+      <c r="D11">
+        <v>17.345315007912301</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="1">
-        <v>1.71755194470252</v>
-      </c>
-      <c r="C12" s="1">
-        <v>1.7178082711451399</v>
-      </c>
-      <c r="D12" s="1">
-        <v>1.7251720106530299</v>
+      <c r="B12">
+        <v>17.154739436798899</v>
+      </c>
+      <c r="C12">
+        <v>17.157242310400498</v>
+      </c>
+      <c r="D12">
+        <v>17.237104830960799</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="1">
-        <v>1.7615745175880899</v>
-      </c>
-      <c r="C13" s="1">
-        <v>1.7614138277217</v>
-      </c>
-      <c r="D13" s="1">
-        <v>1.76809188651991</v>
+      <c r="B13">
+        <v>17.596416562498199</v>
+      </c>
+      <c r="C13">
+        <v>17.5947611027206</v>
+      </c>
+      <c r="D13">
+        <v>17.667195454988001</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -4599,15 +4610,15 @@
       <c r="A18" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="1">
         <f>ABS((C4-C3)/C3)</f>
         <v>0.26819039630949887</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="1">
         <f>ABS((C5-C3)/C3)</f>
         <v>0.31463619207381005</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <f>ABS((C6-C3)/C3)</f>
         <v>0.16177395680436149</v>
       </c>
@@ -4616,27 +4627,27 @@
       <c r="A19" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="1">
         <f>ABS((C11-C10)/C10)</f>
-        <v>6.2170515662932628E-2</v>
-      </c>
-      <c r="C19" s="2">
+        <v>6.2422657438003161E-2</v>
+      </c>
+      <c r="C19" s="1">
         <f>ABS((C12-C10)/C10)</f>
-        <v>6.8121617730053041E-2</v>
-      </c>
-      <c r="D19" s="2">
+        <v>6.8399464023789616E-2</v>
+      </c>
+      <c r="D19" s="1">
         <f>ABS((C13-C10)/C10)</f>
-        <v>4.4466430941682913E-2</v>
+        <v>4.4643155518547271E-2</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="3"/>
+      <c r="C21" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4662,7 +4673,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -4687,92 +4698,92 @@
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3">
-        <v>0.132837940797006</v>
-      </c>
-      <c r="C3">
-        <v>4.71476068422335E-2</v>
-      </c>
-      <c r="D3">
-        <v>4.0631446354482598E-2</v>
-      </c>
-      <c r="E3">
-        <v>6.7857361094004004E-2</v>
+      <c r="B3" s="3">
+        <v>1.3491828990000001</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.47367235699999999</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.40781563900000001</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0.68377695299999997</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B4">
-        <v>0.45704881801401098</v>
-      </c>
-      <c r="C4">
-        <v>0.18438431330628</v>
-      </c>
-      <c r="D4">
-        <v>0.159811500172961</v>
-      </c>
-      <c r="E4">
-        <v>0.259349362226998</v>
+      <c r="B4" s="3">
+        <v>4.5914016670000004</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1.848991979</v>
+      </c>
+      <c r="D4" s="3">
+        <v>1.6018056789999999</v>
+      </c>
+      <c r="E4" s="3">
+        <v>2.6036390140000001</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5">
-        <v>0.70088400530086803</v>
-      </c>
-      <c r="C5">
-        <v>0.34541796582759698</v>
-      </c>
-      <c r="D5">
-        <v>0.30388583540334402</v>
-      </c>
-      <c r="E5">
-        <v>0.46131548553317597</v>
+      <c r="B5" s="3">
+        <v>7.0140517329999996</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.45726975</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3.0412965669999998</v>
+      </c>
+      <c r="E5" s="3">
+        <v>4.6174345839999997</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B6">
-        <v>0.92486510535883804</v>
-      </c>
-      <c r="C6">
-        <v>0.576477041859215</v>
-      </c>
-      <c r="D6">
-        <v>0.52327219067318398</v>
-      </c>
-      <c r="E6">
-        <v>0.70681956698280002</v>
+      <c r="B6" s="3">
+        <v>9.2493070320000008</v>
+      </c>
+      <c r="C6" s="3">
+        <v>5.7607147589999999</v>
+      </c>
+      <c r="D6" s="3">
+        <v>5.229179222</v>
+      </c>
+      <c r="E6" s="3">
+        <v>7.0634611239999998</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
-      <c r="B7">
-        <v>0.43565511996297401</v>
-      </c>
-      <c r="C7">
-        <v>0.43687707375074197</v>
-      </c>
-      <c r="D7">
-        <v>0.43697983419269099</v>
-      </c>
-      <c r="E7">
-        <v>0.43654444642909401</v>
+      <c r="B7" s="3">
+        <v>4.3528580320000003</v>
+      </c>
+      <c r="C7" s="3">
+        <v>4.3642715169999997</v>
+      </c>
+      <c r="D7" s="3">
+        <v>4.3652269190000004</v>
+      </c>
+      <c r="E7" s="3">
+        <v>4.361258791</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="3"/>
+      <c r="B10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
@@ -4792,92 +4803,92 @@
       <c r="A12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <f>ABS((C3-B3)/B3)</f>
-        <v>0.64507424189688922</v>
-      </c>
-      <c r="C12" s="2">
+        <v>0.64891909217713861</v>
+      </c>
+      <c r="C12" s="1">
         <f>ABS((D3-B3)/B3)</f>
-        <v>0.69412770093618936</v>
-      </c>
-      <c r="D12" s="2">
+        <v>0.69773139038282461</v>
+      </c>
+      <c r="D12" s="1">
         <f>ABS((E3-B3)/B3)</f>
-        <v>0.48917183835528544</v>
+        <v>0.49319180260377737</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="1">
         <f>ABS((C4-B4)/B4)</f>
-        <v>0.59657632611878308</v>
-      </c>
-      <c r="C13" s="2">
+        <v>0.59729247992190537</v>
+      </c>
+      <c r="C13" s="1">
         <f>ABS((D4-B4)/B4)</f>
-        <v>0.65034041469053339</v>
-      </c>
-      <c r="D13" s="2">
+        <v>0.65112926396469861</v>
+      </c>
+      <c r="D13" s="1">
         <f>ABS((E4-B4)/B4)</f>
-        <v>0.43255654099722984</v>
+        <v>0.43293155275147049</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="1">
         <f>ABS((C5-B5)/B5)</f>
-        <v>0.50716814306624158</v>
-      </c>
-      <c r="C14" s="2">
+        <v>0.50709377666348043</v>
+      </c>
+      <c r="C14" s="1">
         <f>ABS((D5-B5)/B5)</f>
-        <v>0.56642492465940186</v>
-      </c>
-      <c r="D14" s="2">
+        <v>0.56639946741607528</v>
+      </c>
+      <c r="D14" s="1">
         <f>ABS((E5-B5)/B5)</f>
-        <v>0.34180908389377873</v>
+        <v>0.34168797725347488</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="1">
         <f>ABS((C6-B6)/B6)</f>
-        <v>0.37669067789561816</v>
-      </c>
-      <c r="C15" s="2">
+        <v>0.37717336671065765</v>
+      </c>
+      <c r="C15" s="1">
         <f>ABS((D6-B6)/B6)</f>
-        <v>0.43421782523608154</v>
-      </c>
-      <c r="D15" s="2">
+        <v>0.43464097322010065</v>
+      </c>
+      <c r="D15" s="1">
         <f>ABS((E6-B6)/B6)</f>
-        <v>0.23575928761139564</v>
+        <v>0.23632537015341679</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="1">
         <f>ABS((C7-B7)/B7)</f>
-        <v>2.8048649763873145E-3</v>
-      </c>
-      <c r="C16" s="2">
+        <v>2.6220669077863896E-3</v>
+      </c>
+      <c r="C16" s="1">
         <f>ABS((D7-B7)/B7)</f>
-        <v>3.0407406432628606E-3</v>
-      </c>
-      <c r="D16" s="2">
+        <v>2.8415553434250045E-3</v>
+      </c>
+      <c r="D16" s="1">
         <f>ABS((E7-B7)/B7)</f>
-        <v>2.0413543313701505E-3</v>
+        <v>1.9299409579273184E-3</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="2" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix eval final results
</commit_message>
<xml_diff>
--- a/eval/Final_Results.xlsx
+++ b/eval/Final_Results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ian-g8\projects\FinalTop\eval_10x\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ian-g8\projects\FinalTop\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B361B9F-E226-47A7-9F08-8A33070D0729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C94092A-4D4E-4EFD-A51A-96F9A0D8E433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{DC97868F-0C32-49C4-BD1D-CDEEAEA189B3}"/>
   </bookViews>
@@ -112,8 +112,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -160,100 +161,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="18">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="170" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="170" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="170" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <numFmt numFmtId="170" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0000"/>
+      <numFmt numFmtId="170" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0000"/>
+      <numFmt numFmtId="170" formatCode="0.000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -284,7 +220,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
     </dxf>
     <dxf>
       <font>
@@ -303,7 +239,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
     </dxf>
     <dxf>
       <font>
@@ -322,7 +258,82 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.0%"/>
     </dxf>
     <dxf>
       <font>
@@ -479,19 +490,19 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$B$3:$B$6</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.95379999999999998</c:v>
+                  <c:v>9.5284951539999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.69789999999999996</c:v>
+                  <c:v>6.9729490089999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.65359999999999996</c:v>
+                  <c:v>6.53033866</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.79949999999999999</c:v>
+                  <c:v>7.986455479</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -550,19 +561,19 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$C$3:$C$6</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.95379999999999998</c:v>
+                  <c:v>9.5289460140000006</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.69799999999999995</c:v>
+                  <c:v>6.9738571880000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.65369999999999995</c:v>
+                  <c:v>6.5313767699999996</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.79949999999999999</c:v>
+                  <c:v>7.9871286640000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -621,19 +632,19 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$D$3:$D$6</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.9667</c:v>
+                  <c:v>9.6586474239999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.69720000000000004</c:v>
+                  <c:v>6.9651783140000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.65169999999999995</c:v>
+                  <c:v>6.5110522409999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.80269999999999997</c:v>
+                  <c:v>8.0195223710000008</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -841,7 +852,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1090,7 +1101,7 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$B$10:$B$13</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>18.421462741213698</c:v>
@@ -1161,7 +1172,7 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$C$10:$C$13</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>18.416951952933001</c:v>
@@ -1232,7 +1243,7 @@
             <c:numRef>
               <c:f>Wheel_Gripper_Comparison!$D$10:$D$13</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
                   <c:v>18.475893918431499</c:v>
@@ -1464,7 +1475,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4038,9 +4049,9 @@
   <autoFilter ref="A2:D6" xr:uid="{FCA44438-3D2B-49C3-AEC5-368563795A38}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{10BE39A2-D58C-4415-B31A-E7D54B6146B7}" name="G model"/>
-    <tableColumn id="2" xr3:uid="{82D8A7D9-165E-49C3-9BBA-5C7CCF4E0B90}" name="NH1"/>
-    <tableColumn id="3" xr3:uid="{6FA4CC7A-F19D-4051-8004-C8A708C3ABF0}" name="NH2"/>
-    <tableColumn id="4" xr3:uid="{34A0C971-0CE5-4343-A781-B6485D9A649A}" name="StVK"/>
+    <tableColumn id="2" xr3:uid="{82D8A7D9-165E-49C3-9BBA-5C7CCF4E0B90}" name="NH1" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{6FA4CC7A-F19D-4051-8004-C8A708C3ABF0}" name="NH2" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{34A0C971-0CE5-4343-A781-B6485D9A649A}" name="StVK" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4051,26 +4062,26 @@
   <autoFilter ref="A9:D13" xr:uid="{F98B1F19-8AAE-4F39-9AE7-0F32C71F1F3F}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{72E8BBB5-8A10-4EFF-B75B-A9B4347ABF4C}" name="G model"/>
-    <tableColumn id="2" xr3:uid="{C4C5C7A6-8547-4AA4-B067-90B7D8E52B95}" name="NH1" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{8A9876E2-2BE6-4BFE-9FE6-00BCC5A4596A}" name="NH2" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{D52BB815-B6A5-494E-B26C-07E95A6CF888}" name="StVK" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{C4C5C7A6-8547-4AA4-B067-90B7D8E52B95}" name="NH1" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{8A9876E2-2BE6-4BFE-9FE6-00BCC5A4596A}" name="NH2" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{D52BB815-B6A5-494E-B26C-07E95A6CF888}" name="StVK" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4839363F-B9B0-4E99-BC21-6BC51B855E48}" name="Table5" displayName="Table5" ref="A17:D19" totalsRowShown="0" dataDxfId="3" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4839363F-B9B0-4E99-BC21-6BC51B855E48}" name="Table5" displayName="Table5" ref="A17:D19" totalsRowShown="0" dataDxfId="17" dataCellStyle="Percent">
   <autoFilter ref="A17:D19" xr:uid="{4839363F-B9B0-4E99-BC21-6BC51B855E48}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{B47D74DD-FA03-4401-964F-485ABBC8E85E}" name="Geometry"/>
-    <tableColumn id="2" xr3:uid="{BF908CE0-ED53-49DD-A803-878A9E9653F4}" name="Guth" dataDxfId="2" dataCellStyle="Percent">
+    <tableColumn id="2" xr3:uid="{BF908CE0-ED53-49DD-A803-878A9E9653F4}" name="Guth" dataDxfId="16" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((C10-C9)/C9)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{AF3E19AD-0890-4D34-BDED-1E7928398A92}" name="Mooney" dataDxfId="1" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{AF3E19AD-0890-4D34-BDED-1E7928398A92}" name="Mooney" dataDxfId="15" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((C11-C9)/C9)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC2B6ECF-0580-4856-8BBB-9CF67ABFE4F0}" name="Kerner" dataDxfId="0" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{DC2B6ECF-0580-4856-8BBB-9CF67ABFE4F0}" name="Kerner" dataDxfId="14" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((C12-C9)/C9)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4079,17 +4090,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}" name="Table1" displayName="Table1" ref="A11:D16" totalsRowShown="0" dataDxfId="14" dataCellStyle="Percent">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}" name="Table1" displayName="Table1" ref="A11:D16" totalsRowShown="0" dataDxfId="13" dataCellStyle="Percent">
   <autoFilter ref="A11:D16" xr:uid="{4B7F43FC-C4CD-4ACA-AC46-2B709B2BCAD5}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{1C96DD68-5388-41C8-80A4-631AF2530025}" name="Load Case"/>
-    <tableColumn id="2" xr3:uid="{C0C49FD7-8D17-437F-88C8-BB6258B99219}" name="Guth" dataDxfId="13" dataCellStyle="Percent">
+    <tableColumn id="2" xr3:uid="{C0C49FD7-8D17-437F-88C8-BB6258B99219}" name="Guth" dataDxfId="12" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((C3-B3)/B3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{CB5631BD-80FB-4B0B-BC78-3E45F11C5622}" name="Mooney" dataDxfId="12" dataCellStyle="Percent">
+    <tableColumn id="3" xr3:uid="{CB5631BD-80FB-4B0B-BC78-3E45F11C5622}" name="Mooney" dataDxfId="11" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((D3-B3)/B3)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{64489D84-8154-4AB7-B213-01F3A56C4E26}" name="Kerner" dataDxfId="11" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{64489D84-8154-4AB7-B213-01F3A56C4E26}" name="Kerner" dataDxfId="10" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS((E3-B3)/B3)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4102,10 +4113,10 @@
   <autoFilter ref="A2:E7" xr:uid="{1636F957-79EA-4A9C-A088-0551A65C1F5C}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{BBB9A9AD-3816-4FCF-910B-BC91E45978F8}" name="Load Magnitude"/>
-    <tableColumn id="2" xr3:uid="{C2C97874-87BF-4F49-8E77-46CBD4B4BE4A}" name="Default" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{2269703A-CD27-4542-B024-242B1A805057}" name="Guth" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{CF64BBBD-0D58-4197-9737-466E1D604376}" name="Mooney" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{2F62C0DF-5422-48A6-88EC-800D14AC8CAF}" name="Kerner" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{C2C97874-87BF-4F49-8E77-46CBD4B4BE4A}" name="Default" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{2269703A-CD27-4542-B024-242B1A805057}" name="Guth" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{CF64BBBD-0D58-4197-9737-466E1D604376}" name="Mooney" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{2F62C0DF-5422-48A6-88EC-800D14AC8CAF}" name="Kerner" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4460,56 +4471,56 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3">
-        <v>0.95379999999999998</v>
-      </c>
-      <c r="C3">
-        <v>0.95379999999999998</v>
-      </c>
-      <c r="D3">
-        <v>0.9667</v>
+      <c r="B3" s="4">
+        <v>9.5284951539999998</v>
+      </c>
+      <c r="C3" s="4">
+        <v>9.5289460140000006</v>
+      </c>
+      <c r="D3" s="4">
+        <v>9.6586474239999998</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4">
-        <v>0.69789999999999996</v>
-      </c>
-      <c r="C4">
-        <v>0.69799999999999995</v>
-      </c>
-      <c r="D4">
-        <v>0.69720000000000004</v>
+      <c r="B4" s="4">
+        <v>6.9729490089999997</v>
+      </c>
+      <c r="C4" s="4">
+        <v>6.9738571880000002</v>
+      </c>
+      <c r="D4" s="4">
+        <v>6.9651783140000001</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B5">
-        <v>0.65359999999999996</v>
-      </c>
-      <c r="C5">
-        <v>0.65369999999999995</v>
-      </c>
-      <c r="D5">
-        <v>0.65169999999999995</v>
+      <c r="B5" s="4">
+        <v>6.53033866</v>
+      </c>
+      <c r="C5" s="4">
+        <v>6.5313767699999996</v>
+      </c>
+      <c r="D5" s="4">
+        <v>6.5110522409999998</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
-        <v>0.79949999999999999</v>
-      </c>
-      <c r="C6">
-        <v>0.79949999999999999</v>
-      </c>
-      <c r="D6">
-        <v>0.80269999999999997</v>
+      <c r="B6" s="4">
+        <v>7.986455479</v>
+      </c>
+      <c r="C6" s="4">
+        <v>7.9871286640000001</v>
+      </c>
+      <c r="D6" s="4">
+        <v>8.0195223710000008</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -4535,13 +4546,13 @@
       <c r="A10" t="s">
         <v>4</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="4">
         <v>18.421462741213698</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="4">
         <v>18.416951952933001</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="4">
         <v>18.475893918431499</v>
       </c>
     </row>
@@ -4549,13 +4560,13 @@
       <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="4">
         <v>17.266254811593701</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="4">
         <v>17.267316870122901</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="4">
         <v>17.345315007912301</v>
       </c>
     </row>
@@ -4563,13 +4574,13 @@
       <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="4">
         <v>17.154739436798899</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="4">
         <v>17.157242310400498</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="4">
         <v>17.237104830960799</v>
       </c>
     </row>
@@ -4577,13 +4588,13 @@
       <c r="A13" t="s">
         <v>7</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="4">
         <v>17.596416562498199</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="4">
         <v>17.5947611027206</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="4">
         <v>17.667195454988001</v>
       </c>
     </row>
@@ -4612,15 +4623,15 @@
       </c>
       <c r="B18" s="1">
         <f>ABS((C4-C3)/C3)</f>
-        <v>0.26819039630949887</v>
+        <v>0.26813971054574604</v>
       </c>
       <c r="C18" s="1">
         <f>ABS((C5-C3)/C3)</f>
-        <v>0.31463619207381005</v>
+        <v>0.31457511036330243</v>
       </c>
       <c r="D18" s="1">
         <f>ABS((C6-C3)/C3)</f>
-        <v>0.16177395680436149</v>
+        <v>0.16180355600029117</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>